<commit_message>
Update 2026 League scoresheet and annual calendar data files
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/HHBClubAnnualCalendar.xlsx
+++ b/data/HHBClubAnnualCalendar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/22393d3a424cfc66/badminton_club_app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_27EC31309C5DEF86491B0751F0D96019553E0DB4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0583B8CC-E600-4546-8077-E4A0547821BA}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="11_27EC31309C5DEF86491B0751F0D96019553E0DB4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D5157D0-A407-4C03-914C-9CDE0D698628}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>HHB Club Annual Calendar</t>
   </si>
@@ -97,16 +97,6 @@
     <t>7 &amp; 14 Jun</t>
   </si>
   <si>
-    <t>As every year ... (missed out in 2025)
-No player sign up or no limits - everybody participates by default.
-Players report all match scores every Sunday. 
-Ranking League table based on reported matches.
-(Individuals can opt out of the League Table if they wish to)
-Top of the Table after 10 weeks get trophies.
-Winner, Runner Up and 3rd Place gets trophies.
-3 Trophies up for grabs.</t>
-  </si>
-  <si>
     <t>10 weeks from Sep-Nov
 5 Sundays before October School Holidays
 5 Sundays after October School Holidays</t>
@@ -143,6 +133,19 @@
 Pool B players randomly pair within the Pool and compete. 
 Winner and Runner Ups from both Pools get trophies.
 8 Trophies up for grabs !</t>
+  </si>
+  <si>
+    <t>6 &amp; 13th June</t>
+  </si>
+  <si>
+    <t>As every year ... (missed out in 2025)
+No player sign up or no limits - everybody participates by default.
+Players report all match scores every Sunday. 
+Players League table based on reported matches.
+(Individuals can opt out of the League Table if they wish to)
+Top of the Table after 10 weeks get trophies.
+Winner, Runner Up and 3rd Place gets trophies.
+3 Trophies up for grabs.</t>
   </si>
 </sst>
 </file>
@@ -383,39 +386,64 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -639,146 +667,150 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="59.25" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.5703125" customWidth="1"/>
-    <col min="2" max="2" width="40.28515625" customWidth="1"/>
-    <col min="3" max="3" width="81.140625" customWidth="1"/>
-    <col min="4" max="4" width="48.7109375" customWidth="1"/>
-    <col min="5" max="5" width="24.28515625" customWidth="1"/>
+    <col min="2" max="2" width="45" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="81.140625" style="13" customWidth="1"/>
+    <col min="4" max="4" width="48.7109375" style="13" customWidth="1"/>
+    <col min="5" max="5" width="24.28515625" style="13" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
     </row>
-    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:6" ht="50.25" x14ac:dyDescent="0.7">
       <c r="A2" s="1"/>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="23"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="11"/>
     </row>
-    <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="16" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8" t="s">
+    <row r="4" spans="1:6" ht="132.75" x14ac:dyDescent="0.35">
+      <c r="A4" s="4"/>
+      <c r="B4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A5" s="4"/>
+      <c r="B5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A6" s="4"/>
+      <c r="B6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="20">
+        <v>46136</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="151.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="4"/>
+      <c r="B7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>9</v>
-      </c>
     </row>
-    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="7"/>
-      <c r="B5" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>14</v>
+    <row r="8" spans="1:6" ht="170.25" x14ac:dyDescent="0.35">
+      <c r="A8" s="4"/>
+      <c r="B8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="7"/>
-      <c r="B6" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="14">
-        <v>46136</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="7"/>
-      <c r="B7" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="7"/>
-      <c r="B8" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="17" t="s">
+    <row r="9" spans="1:6" ht="59.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4"/>
+      <c r="B9" s="8" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="7"/>
-      <c r="B9" s="18" t="s">
+      <c r="C9" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="D9" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="E9" s="24" t="s">
         <v>27</v>
-      </c>
-      <c r="E9" s="20" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>